<commit_message>
Fix Uzbek apostrophes in Excel template directly
- Y column IF formulas: U+2019/U+2018 → U+02BC (aʼlo), U+02BB (oʻrta, qoʻyilmadi)
- COUNTIF formulas: same fix — now Y values and COUNTIF criteria match
- Remove PHP workaround from JournalController (no longer needed)

https://claude.ai/code/session_01PphoiJYfSyExEEu5nZPKMD
</commit_message>
<xml_diff>
--- a/public/templates/yn_qaydnoma (1).xlsx
+++ b/public/templates/yn_qaydnoma (1).xlsx
@@ -4048,7 +4048,7 @@
       </c>
       <c r="X20" s="5"/>
       <c r="Y20" s="5" t="str">
-        <f>IF(B20=0,"",IF((V20&gt;=90)*(V20&lt;=100),"a’lo",IF((V20&gt;=70)*(V20&lt;=89.9),"yaxshi",IF((V20&gt;=60)*(V20&lt;=69.9),"o‘rta",IF((V20&gt;=0)*(V20&lt;=59.9),"qon-siz",IF(V20=-1,"kelmadi",IF(V20=-2,"qo‘yilmadi","")))))))</f>
+        <f>IF(B20=0,"",IF((V20&gt;=90)*(V20&lt;=100),"aʼlo",IF((V20&gt;=70)*(V20&lt;=89.9),"yaxshi",IF((V20&gt;=60)*(V20&lt;=69.9),"oʻrta",IF((V20&gt;=0)*(V20&lt;=59.9),"qon-siz",IF(V20=-1,"kelmadi",IF(V20=-2,"qoʻyilmadi","")))))))</f>
         <v/>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       </c>
       <c r="X21" s="6"/>
       <c r="Y21" s="6" t="str">
-        <f t="shared" ref="Y21:Y49" si="9">IF(B21=0,"",IF((V21&gt;=90)*(V21&lt;=100),"a’lo",IF((V21&gt;=70)*(V21&lt;=89.9),"yaxshi",IF((V21&gt;=60)*(V21&lt;=69.9),"o‘rta",IF((V21&gt;=0)*(V21&lt;=59.9),"qon-siz",IF(V21=-1,"kelmadi",IF(V21=-2,"qo‘yilmadi","")))))))</f>
+        <f t="shared" ref="Y21:Y49" si="9">IF(B21=0,"",IF((V21&gt;=90)*(V21&lt;=100),"aʼlo",IF((V21&gt;=70)*(V21&lt;=89.9),"yaxshi",IF((V21&gt;=60)*(V21&lt;=69.9),"oʻrta",IF((V21&gt;=0)*(V21&lt;=59.9),"qon-siz",IF(V21=-1,"kelmadi",IF(V21=-2,"qoʻyilmadi","")))))))</f>
         <v/>
       </c>
     </row>
@@ -5909,7 +5909,7 @@
       </c>
       <c r="E57" s="174"/>
       <c r="F57" s="173">
-        <f>COUNTIF(Y20:Y49,"a‘lo")</f>
+        <f>COUNTIF(Y20:Y49,"aʼlo")</f>
         <v>0</v>
       </c>
       <c r="G57" s="174"/>
@@ -5924,7 +5924,7 @@
       <c r="L57" s="176"/>
       <c r="M57" s="177"/>
       <c r="N57" s="11">
-        <f>COUNTIF(Y20:Y49,"o‘rta")</f>
+        <f>COUNTIF(Y20:Y49,"oʻrta")</f>
         <v>0</v>
       </c>
       <c r="O57" s="12"/>
@@ -5984,7 +5984,7 @@
       <c r="T58" s="178"/>
       <c r="U58" s="178"/>
       <c r="V58" s="13">
-        <f>COUNTIF(Y20:Y49,"qo‘yilmadi")</f>
+        <f>COUNTIF(Y20:Y49,"qoʻyilmadi")</f>
         <v>0</v>
       </c>
       <c r="W58" s="75">

</xml_diff>